<commit_message>
started restructuring for thesis hand-in
</commit_message>
<xml_diff>
--- a/Tasks.xlsx
+++ b/Tasks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\Documents\David\Unibe\MT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60294929-5A19-49E4-97F9-E5EE3D59096A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D5788DA-75D8-4455-AF11-5B822A6B5015}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-3900" yWindow="-17388" windowWidth="41496" windowHeight="16776" xr2:uid="{C826B7FA-C91E-4397-A3F1-6A59F949C2CD}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" xr2:uid="{C826B7FA-C91E-4397-A3F1-6A59F949C2CD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="39">
   <si>
     <t>Task</t>
   </si>
@@ -110,9 +110,6 @@
     <t>M, R</t>
   </si>
   <si>
-    <t>Review M + R</t>
-  </si>
-  <si>
     <t>Write Conclusion</t>
   </si>
   <si>
@@ -122,18 +119,9 @@
     <t>Conclusion</t>
   </si>
   <si>
-    <t>Review I + M</t>
-  </si>
-  <si>
-    <t>Review R + D + C</t>
-  </si>
-  <si>
     <t>Review Everything</t>
   </si>
   <si>
-    <t>I, M</t>
-  </si>
-  <si>
     <t>all</t>
   </si>
   <si>
@@ -150,6 +138,21 @@
   </si>
   <si>
     <t>Add Objective to I</t>
+  </si>
+  <si>
+    <t>Review R + D</t>
+  </si>
+  <si>
+    <t>R, D</t>
+  </si>
+  <si>
+    <t>Revise Discussion</t>
+  </si>
+  <si>
+    <t>GitHub Repository</t>
+  </si>
+  <si>
+    <t>Review Data section</t>
   </si>
 </sst>
 </file>
@@ -749,7 +752,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB665F84-8968-4167-86A1-2FFD61C43281}">
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="13.59765625" customWidth="1"/>
@@ -816,7 +819,7 @@
         <v>46083</v>
       </c>
       <c r="B4" s="2" t="str">
-        <f t="shared" ref="B4:B24" si="0">TEXT(A4,"dddd")</f>
+        <f t="shared" ref="B4:B25" si="0">TEXT(A4,"dddd")</f>
         <v>Monday</v>
       </c>
       <c r="C4" s="3" t="s">
@@ -910,7 +913,7 @@
         <v>Friday</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>11</v>
@@ -1018,12 +1021,14 @@
         <v>Wednesday</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E15" s="4"/>
+        <v>30</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="16" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="1">
@@ -1037,9 +1042,11 @@
         <v>21</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E16" s="4"/>
+        <v>30</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="17" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="1">
@@ -1050,30 +1057,34 @@
         <v>Thursday</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E17" s="4"/>
+        <v>35</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="18" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="1">
         <v>46094</v>
       </c>
       <c r="B18" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="B18" si="3">TEXT(A18,"dddd")</f>
         <v>Friday</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E18" s="4"/>
-    </row>
-    <row r="19" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.45">
+        <v>10</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="1">
         <v>46095</v>
       </c>
@@ -1082,44 +1093,50 @@
         <v>Saturday</v>
       </c>
       <c r="C19" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E19" s="4"/>
+      <c r="E19" s="4" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="20" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="1">
         <v>46096</v>
       </c>
       <c r="B20" s="2" t="str">
-        <f t="shared" ref="B20" si="3">TEXT(A20,"dddd")</f>
+        <f t="shared" si="0"/>
         <v>Sunday</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="E20" s="4"/>
+        <v>26</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="21" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="1">
-        <v>46096</v>
+        <v>46097</v>
       </c>
       <c r="B21" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>Sunday</v>
+        <f t="shared" ref="B21" si="4">TEXT(A21,"dddd")</f>
+        <v>Monday</v>
       </c>
       <c r="C21" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D21" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E21" s="4"/>
+      <c r="E21" s="4" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="22" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="1">
@@ -1130,10 +1147,10 @@
         <v>Monday</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E22" s="4"/>
     </row>
@@ -1146,30 +1163,46 @@
         <v>Tuesday</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E23" s="4"/>
     </row>
     <row r="24" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="1">
+        <v>46098</v>
+      </c>
+      <c r="B24" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>Tuesday</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E24" s="4"/>
+    </row>
+    <row r="25" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A25" s="1">
         <v>46099</v>
       </c>
-      <c r="B24" s="2" t="str">
+      <c r="B25" s="2" t="str">
         <f t="shared" si="0"/>
         <v>Wednesday</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C25" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D24" s="2"/>
-      <c r="E24" s="4"/>
+      <c r="D25" s="2"/>
+      <c r="E25" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="A1:E24">
+  <conditionalFormatting sqref="A1:E25">
     <cfRule type="expression" dxfId="8" priority="3">
       <formula>WEEKDAY($A1)=1</formula>
     </cfRule>
@@ -1192,7 +1225,7 @@
       <formula>WEEKDAY($A1)=7</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E24">
+  <conditionalFormatting sqref="E2:E25">
     <cfRule type="expression" dxfId="1" priority="1">
       <formula>$E2="Delayed"</formula>
     </cfRule>

</xml_diff>